<commit_message>
feat: agrega excedentes y hoja Resumen
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="53">
   <si>
     <t xml:space="preserve">Código</t>
   </si>
@@ -41,6 +42,9 @@
     <t xml:space="preserve">Stock máximo</t>
   </si>
   <si>
+    <t xml:space="preserve">Excedente (unid.)</t>
+  </si>
+  <si>
     <t xml:space="preserve">REP-001</t>
   </si>
   <si>
@@ -165,16 +169,29 @@
   </si>
   <si>
     <t xml:space="preserve">Regla: Stock actual = 0 es SIN STOCK; menor al mínimo es REPONER; mayor al máximo es excedente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen de inventario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total de productos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productos con excedente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidades en exceso (total)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,6 +238,13 @@
     <font>
       <b val="true"/>
       <sz val="13"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -289,7 +313,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -306,11 +330,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -323,6 +355,15 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -360,7 +401,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -566,13 +607,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -594,16 +636,19 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0</v>
@@ -614,16 +659,20 @@
       <c r="F2" s="3" t="n">
         <v>80</v>
       </c>
+      <c r="G2" s="4" t="n">
+        <f aca="false">MAX(0,D2-F2)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>35</v>
@@ -634,16 +683,20 @@
       <c r="F3" s="3" t="n">
         <v>80</v>
       </c>
+      <c r="G3" s="4" t="n">
+        <f aca="false">MAX(0,D3-F3)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>12</v>
@@ -654,16 +707,20 @@
       <c r="F4" s="3" t="n">
         <v>40</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <f aca="false">MAX(0,D4-F4)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>150</v>
@@ -674,16 +731,20 @@
       <c r="F5" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="G5" s="4" t="n">
+        <f aca="false">MAX(0,D5-F5)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>18</v>
@@ -694,16 +755,20 @@
       <c r="F6" s="3" t="n">
         <v>90</v>
       </c>
+      <c r="G6" s="4" t="n">
+        <f aca="false">MAX(0,D6-F6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0</v>
@@ -714,16 +779,20 @@
       <c r="F7" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="G7" s="4" t="n">
+        <f aca="false">MAX(0,D7-F7)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>6</v>
@@ -734,16 +803,20 @@
       <c r="F8" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="G8" s="4" t="n">
+        <f aca="false">MAX(0,D8-F8)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>44</v>
@@ -754,16 +827,20 @@
       <c r="F9" s="3" t="n">
         <v>40</v>
       </c>
+      <c r="G9" s="4" t="n">
+        <f aca="false">MAX(0,D9-F9)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>60</v>
@@ -774,16 +851,20 @@
       <c r="F10" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="G10" s="4" t="n">
+        <f aca="false">MAX(0,D10-F10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>9</v>
@@ -794,16 +875,20 @@
       <c r="F11" s="3" t="n">
         <v>30</v>
       </c>
+      <c r="G11" s="4" t="n">
+        <f aca="false">MAX(0,D11-F11)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>3</v>
@@ -814,16 +899,20 @@
       <c r="F12" s="3" t="n">
         <v>35</v>
       </c>
+      <c r="G12" s="4" t="n">
+        <f aca="false">MAX(0,D12-F12)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>25</v>
@@ -834,16 +923,20 @@
       <c r="F13" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="G13" s="4" t="n">
+        <f aca="false">MAX(0,D13-F13)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
@@ -854,16 +947,20 @@
       <c r="F14" s="3" t="n">
         <v>25</v>
       </c>
+      <c r="G14" s="4" t="n">
+        <f aca="false">MAX(0,D14-F14)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>7</v>
@@ -874,16 +971,20 @@
       <c r="F15" s="3" t="n">
         <v>15</v>
       </c>
+      <c r="G15" s="4" t="n">
+        <f aca="false">MAX(0,D15-F15)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>90</v>
@@ -894,8 +995,17 @@
       <c r="F16" s="3" t="n">
         <v>60</v>
       </c>
+      <c r="G16" s="4" t="n">
+        <f aca="false">MAX(0,D16-F16)</f>
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G2:G16">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -918,28 +1028,83 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>43</v>
+      <c r="A1" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>44</v>
+      <c r="A2" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>45</v>
+      <c r="A3" s="6" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>46</v>
+      <c r="A4" s="6" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>47</v>
+      <c r="A5" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <f aca="false">COUNTA(Inventario!A2:A16)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <f aca="false">COUNTIF(Inventario!G2:G16,"&gt;0")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <f aca="false">SUM(Inventario!G2:G16)</f>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: agrega columna Estado (SIN STOCK / REPONER / OK)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="49">
   <si>
     <t xml:space="preserve">Código</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t xml:space="preserve">Stock máximo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado</t>
   </si>
   <si>
     <t xml:space="preserve">REP-001</t>
@@ -174,7 +177,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +217,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -289,7 +299,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -306,7 +316,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -323,6 +337,29 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -359,12 +396,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFC6E0B4"/>
+      <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFF8CBAD"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -566,13 +603,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -594,16 +632,19 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0</v>
@@ -614,16 +655,20 @@
       <c r="F2" s="3" t="n">
         <v>80</v>
       </c>
+      <c r="G2" s="4" t="str">
+        <f aca="false">IF(D2=0,"SIN STOCK",IF(D2&lt;E2,"REPONER","OK"))</f>
+        <v>SIN STOCK</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>35</v>
@@ -634,16 +679,20 @@
       <c r="F3" s="3" t="n">
         <v>80</v>
       </c>
+      <c r="G3" s="4" t="str">
+        <f aca="false">IF(D3=0,"SIN STOCK",IF(D3&lt;E3,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>12</v>
@@ -654,16 +703,20 @@
       <c r="F4" s="3" t="n">
         <v>40</v>
       </c>
+      <c r="G4" s="4" t="str">
+        <f aca="false">IF(D4=0,"SIN STOCK",IF(D4&lt;E4,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>150</v>
@@ -674,16 +727,20 @@
       <c r="F5" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="G5" s="4" t="str">
+        <f aca="false">IF(D5=0,"SIN STOCK",IF(D5&lt;E5,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>18</v>
@@ -694,16 +751,20 @@
       <c r="F6" s="3" t="n">
         <v>90</v>
       </c>
+      <c r="G6" s="4" t="str">
+        <f aca="false">IF(D6=0,"SIN STOCK",IF(D6&lt;E6,"REPONER","OK"))</f>
+        <v>REPONER</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0</v>
@@ -714,16 +775,20 @@
       <c r="F7" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="G7" s="4" t="str">
+        <f aca="false">IF(D7=0,"SIN STOCK",IF(D7&lt;E7,"REPONER","OK"))</f>
+        <v>SIN STOCK</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>6</v>
@@ -734,16 +799,20 @@
       <c r="F8" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="G8" s="4" t="str">
+        <f aca="false">IF(D8=0,"SIN STOCK",IF(D8&lt;E8,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>44</v>
@@ -754,16 +823,20 @@
       <c r="F9" s="3" t="n">
         <v>40</v>
       </c>
+      <c r="G9" s="4" t="str">
+        <f aca="false">IF(D9=0,"SIN STOCK",IF(D9&lt;E9,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>60</v>
@@ -774,16 +847,20 @@
       <c r="F10" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="G10" s="4" t="str">
+        <f aca="false">IF(D10=0,"SIN STOCK",IF(D10&lt;E10,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>9</v>
@@ -794,16 +871,20 @@
       <c r="F11" s="3" t="n">
         <v>30</v>
       </c>
+      <c r="G11" s="4" t="str">
+        <f aca="false">IF(D11=0,"SIN STOCK",IF(D11&lt;E11,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>3</v>
@@ -814,16 +895,20 @@
       <c r="F12" s="3" t="n">
         <v>35</v>
       </c>
+      <c r="G12" s="4" t="str">
+        <f aca="false">IF(D12=0,"SIN STOCK",IF(D12&lt;E12,"REPONER","OK"))</f>
+        <v>REPONER</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>25</v>
@@ -834,16 +919,20 @@
       <c r="F13" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="G13" s="4" t="str">
+        <f aca="false">IF(D13=0,"SIN STOCK",IF(D13&lt;E13,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
@@ -854,16 +943,20 @@
       <c r="F14" s="3" t="n">
         <v>25</v>
       </c>
+      <c r="G14" s="4" t="str">
+        <f aca="false">IF(D14=0,"SIN STOCK",IF(D14&lt;E14,"REPONER","OK"))</f>
+        <v>SIN STOCK</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>7</v>
@@ -874,16 +967,20 @@
       <c r="F15" s="3" t="n">
         <v>15</v>
       </c>
+      <c r="G15" s="4" t="str">
+        <f aca="false">IF(D15=0,"SIN STOCK",IF(D15&lt;E15,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>90</v>
@@ -894,8 +991,23 @@
       <c r="F16" s="3" t="n">
         <v>60</v>
       </c>
+      <c r="G16" s="4" t="str">
+        <f aca="false">IF(D16=0,"SIN STOCK",IF(D16&lt;E16,"REPONER","OK"))</f>
+        <v>OK</v>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G2:G16">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"SIN STOCK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"REPONER"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -918,28 +1030,28 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>43</v>
+      <c r="A1" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>44</v>
+      <c r="A2" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>45</v>
+      <c r="A3" s="6" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>46</v>
+      <c r="A4" s="6" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>47</v>
+      <c r="A5" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>